<commit_message>
Semana 09: Ajustar tabla de evidencias a 2x3 para organizar los 5 intentos y resumen en Docs
</commit_message>
<xml_diff>
--- a/assets/semana09/Kahoot_Semana09_CulturaDigital.xlsx
+++ b/assets/semana09/Kahoot_Semana09_CulturaDigital.xlsx
@@ -959,12 +959,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>¿Por qué insertamos una tabla de 2x1 para pegar la captura de pantalla?</t>
+          <t>¿Por qué insertamos una tabla de 2x3 para pegar las capturas de pantalla?</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Para evitar que la imagen gigante desborde o mueva el texto</t>
+          <t>Para evitar que las imágenes gigantes desborden o muevan el texto</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">

</xml_diff>